<commit_message>
temporary fix to SYVBT to adjust allocation of freight HDVs (previously 99% gas, switched to diesel)
</commit_message>
<xml_diff>
--- a/InputData/trans/SYVbT/Start Year Vehicles by Technology.xlsx
+++ b/InputData/trans/SYVbT/Start Year Vehicles by Technology.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\Mexico EPS\InputData\trans\SYVbT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\eps-mexico\InputData\trans\SYVbT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ADCFEE3-EE4F-421D-9E7F-B8BB47F83F39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF67BB43-7868-42EA-92BA-F47C9CCA543F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44145" yWindow="1230" windowWidth="22785" windowHeight="14115" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -4365,7 +4365,16 @@
     <xf numFmtId="0" fontId="49" fillId="2" borderId="0" xfId="73" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="73" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="36" borderId="21" xfId="73" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="60" fillId="36" borderId="0" xfId="73" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="61" fillId="37" borderId="0" xfId="73" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="73" applyFont="1"/>
@@ -4373,14 +4382,23 @@
     <xf numFmtId="0" fontId="57" fillId="35" borderId="23" xfId="73" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="73" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="36" borderId="21" xfId="73" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="61" fillId="37" borderId="0" xfId="73" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -4389,25 +4407,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
@@ -5664,9 +5664,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B38"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="73.109375" customWidth="1"/>
+    <col min="2" max="2" width="73.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -5849,15 +5849,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA9ECEC9-2D67-2F44-9D1D-E497A821C590}">
   <dimension ref="A1:AU81"/>
-  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30.88671875" style="69" customWidth="1"/>
-    <col min="2" max="2" width="11.109375" style="69" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.88671875" style="69"/>
-    <col min="4" max="4" width="13.6640625" style="69" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="11.109375" style="69" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.85546875" style="69" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" style="69" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" style="69"/>
+    <col min="4" max="4" width="13.7109375" style="69" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.140625" style="69" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="11" style="69" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="10.88671875" style="69"/>
+    <col min="9" max="16384" width="10.85546875" style="69"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:47">
@@ -7457,12 +7457,11 @@
         <v>2.9494640303658694E-4</v>
       </c>
       <c r="D69" s="69">
-        <f t="shared" si="5"/>
-        <v>0.97655269722388449</v>
+        <f>1-SUM(B69:C69,E69:H69)</f>
+        <v>1.4676144350825204E-2</v>
       </c>
       <c r="E69" s="69">
-        <f t="shared" si="5"/>
-        <v>1.8123447126940927E-2</v>
+        <v>0.98</v>
       </c>
       <c r="G69" s="69">
         <f t="shared" si="5"/>
@@ -7513,11 +7512,11 @@
       </c>
       <c r="D71" s="5">
         <f t="shared" si="6"/>
-        <v>1747052.7753335293</v>
+        <v>26255.622243626291</v>
       </c>
       <c r="E71" s="5">
-        <f t="shared" si="6"/>
-        <v>32422.84691009732</v>
+        <f>$B46*E$69</f>
+        <v>1753220</v>
       </c>
       <c r="F71" s="5">
         <f t="shared" si="6"/>
@@ -7546,11 +7545,11 @@
       </c>
       <c r="D72" s="5">
         <f t="shared" si="6"/>
-        <v>606439.22497603227</v>
+        <v>9113.8856418624528</v>
       </c>
       <c r="E72" s="5">
-        <f t="shared" si="6"/>
-        <v>11254.660665830315</v>
+        <f>$B47*E$69</f>
+        <v>608580</v>
       </c>
       <c r="F72" s="84">
         <f t="shared" si="6"/>
@@ -7886,7 +7885,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{847F86A9-3044-3740-AA01-A50E40D8D85E}">
   <dimension ref="B26:F30"/>
-  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <sheetData>
     <row r="26" spans="2:6">
       <c r="B26" t="s">
@@ -7938,15 +7937,15 @@
     <tabColor theme="1" tint="0.34998626667073579"/>
   </sheetPr>
   <dimension ref="A2:AL409"/>
-  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="2" style="32" customWidth="1"/>
-    <col min="3" max="3" width="23.109375" style="32" customWidth="1"/>
+    <col min="3" max="3" width="23.140625" style="32" customWidth="1"/>
     <col min="4" max="4" width="33" style="32" bestFit="1" customWidth="1"/>
-    <col min="5" max="36" width="6.33203125" style="32" customWidth="1"/>
-    <col min="37" max="37" width="7.6640625" style="32" customWidth="1"/>
+    <col min="5" max="36" width="6.28515625" style="32" customWidth="1"/>
+    <col min="37" max="37" width="7.7109375" style="32" customWidth="1"/>
     <col min="38" max="38" width="2" style="32" customWidth="1"/>
-    <col min="39" max="16384" width="11.44140625" style="32"/>
+    <col min="39" max="16384" width="11.42578125" style="32"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:38">
@@ -8224,46 +8223,46 @@
       </c>
     </row>
     <row r="5" spans="1:38" ht="13.5" customHeight="1">
-      <c r="A5" s="93" t="s">
+      <c r="A5" s="89" t="s">
         <v>114</v>
       </c>
-      <c r="B5" s="93"/>
-      <c r="C5" s="93"/>
-      <c r="D5" s="93"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
-      <c r="I5" s="93"/>
-      <c r="J5" s="93"/>
-      <c r="K5" s="93"/>
-      <c r="L5" s="93"/>
-      <c r="M5" s="93"/>
-      <c r="N5" s="93"/>
-      <c r="O5" s="93"/>
-      <c r="P5" s="93"/>
-      <c r="Q5" s="93"/>
-      <c r="R5" s="93"/>
-      <c r="S5" s="93"/>
-      <c r="T5" s="93"/>
-      <c r="U5" s="93"/>
-      <c r="V5" s="93"/>
-      <c r="W5" s="93"/>
-      <c r="X5" s="93"/>
-      <c r="Y5" s="93"/>
-      <c r="Z5" s="93"/>
-      <c r="AA5" s="93"/>
-      <c r="AB5" s="93"/>
-      <c r="AC5" s="93"/>
-      <c r="AD5" s="93"/>
-      <c r="AE5" s="93"/>
-      <c r="AF5" s="93"/>
-      <c r="AG5" s="93"/>
-      <c r="AH5" s="93"/>
-      <c r="AI5" s="93"/>
-      <c r="AJ5" s="93"/>
-      <c r="AK5" s="93"/>
-      <c r="AL5" s="93"/>
+      <c r="B5" s="89"/>
+      <c r="C5" s="89"/>
+      <c r="D5" s="89"/>
+      <c r="E5" s="89"/>
+      <c r="F5" s="89"/>
+      <c r="G5" s="89"/>
+      <c r="H5" s="89"/>
+      <c r="I5" s="89"/>
+      <c r="J5" s="89"/>
+      <c r="K5" s="89"/>
+      <c r="L5" s="89"/>
+      <c r="M5" s="89"/>
+      <c r="N5" s="89"/>
+      <c r="O5" s="89"/>
+      <c r="P5" s="89"/>
+      <c r="Q5" s="89"/>
+      <c r="R5" s="89"/>
+      <c r="S5" s="89"/>
+      <c r="T5" s="89"/>
+      <c r="U5" s="89"/>
+      <c r="V5" s="89"/>
+      <c r="W5" s="89"/>
+      <c r="X5" s="89"/>
+      <c r="Y5" s="89"/>
+      <c r="Z5" s="89"/>
+      <c r="AA5" s="89"/>
+      <c r="AB5" s="89"/>
+      <c r="AC5" s="89"/>
+      <c r="AD5" s="89"/>
+      <c r="AE5" s="89"/>
+      <c r="AF5" s="89"/>
+      <c r="AG5" s="89"/>
+      <c r="AH5" s="89"/>
+      <c r="AI5" s="89"/>
+      <c r="AJ5" s="89"/>
+      <c r="AK5" s="89"/>
+      <c r="AL5" s="89"/>
     </row>
     <row r="6" spans="1:38" ht="13.5" customHeight="1" thickBot="1"/>
     <row r="7" spans="1:38" s="62" customFormat="1" ht="22.5" customHeight="1" thickTop="1" thickBot="1">
@@ -8376,10 +8375,10 @@
     </row>
     <row r="8" spans="1:38" s="62" customFormat="1" ht="21" customHeight="1" thickTop="1">
       <c r="B8" s="61"/>
-      <c r="C8" s="94" t="s">
+      <c r="C8" s="90" t="s">
         <v>117</v>
       </c>
-      <c r="D8" s="94"/>
+      <c r="D8" s="90"/>
       <c r="E8" s="60">
         <f t="shared" ref="E8:AJ8" si="2">+E9+E14+E23+E18+E40+E42+E62+E75+E79+E82+E95+E102+E119+E121</f>
         <v>130</v>
@@ -13501,10 +13500,10 @@
       <c r="B93" s="55">
         <v>6</v>
       </c>
-      <c r="C93" s="95" t="s">
+      <c r="C93" s="92" t="s">
         <v>193</v>
       </c>
-      <c r="D93" s="95"/>
+      <c r="D93" s="92"/>
       <c r="E93" s="54"/>
       <c r="F93" s="54"/>
       <c r="G93" s="54"/>
@@ -15377,10 +15376,10 @@
     </row>
     <row r="129" spans="2:37" ht="21" customHeight="1">
       <c r="B129" s="61"/>
-      <c r="C129" s="89" t="s">
+      <c r="C129" s="91" t="s">
         <v>218</v>
       </c>
-      <c r="D129" s="89"/>
+      <c r="D129" s="91"/>
       <c r="E129" s="60">
         <f t="shared" ref="E129:AJ129" si="14">+E130+E134+E137+E139+E144+E158+E162+E164+E167+E173+E179+E190+E193+E198+E202+E213+E215+E217+E220+E225</f>
         <v>54</v>
@@ -20936,10 +20935,10 @@
     </row>
     <row r="228" spans="2:37" ht="21" customHeight="1">
       <c r="B228" s="61"/>
-      <c r="C228" s="89" t="s">
+      <c r="C228" s="91" t="s">
         <v>288</v>
       </c>
-      <c r="D228" s="89"/>
+      <c r="D228" s="91"/>
       <c r="E228" s="60">
         <f t="shared" ref="E228:AJ228" si="27">+E229+E231+E234+E237+E240+E242+E244+E247+E249+E251+E253+E255+E257+E268+E270+E275+E277+E279+E281+E289</f>
         <v>4</v>
@@ -24015,10 +24014,10 @@
     </row>
     <row r="291" spans="2:37" ht="21" customHeight="1">
       <c r="B291" s="61"/>
-      <c r="C291" s="89" t="s">
+      <c r="C291" s="91" t="s">
         <v>323</v>
       </c>
-      <c r="D291" s="89"/>
+      <c r="D291" s="91"/>
       <c r="E291" s="60"/>
       <c r="F291" s="60">
         <f t="shared" ref="F291:AJ291" si="31">+F292+F294+F296+F299+F301+F304+F306+F309+F315+F331+F335+F337+F346+F348+F351+F362+F365+F367+F370+F372+F375+F379+F384+F386+F390+F396</f>
@@ -30128,10 +30127,10 @@
     </row>
     <row r="403" spans="2:38" s="37" customFormat="1" ht="22.5" customHeight="1" thickTop="1" thickBot="1">
       <c r="B403" s="42"/>
-      <c r="C403" s="92" t="s">
+      <c r="C403" s="95" t="s">
         <v>419</v>
       </c>
-      <c r="D403" s="92"/>
+      <c r="D403" s="95"/>
       <c r="E403" s="40">
         <f t="shared" ref="E403:AK403" si="49">+E291+E228+E129+E8</f>
         <v>188</v>
@@ -30270,10 +30269,10 @@
       <c r="B404" s="35" t="s">
         <v>420</v>
       </c>
-      <c r="C404" s="91" t="s">
+      <c r="C404" s="94" t="s">
         <v>421</v>
       </c>
-      <c r="D404" s="91"/>
+      <c r="D404" s="94"/>
       <c r="AC404" s="36"/>
       <c r="AD404" s="36"/>
       <c r="AE404" s="36"/>
@@ -30287,28 +30286,28 @@
       <c r="B405" s="35" t="s">
         <v>422</v>
       </c>
-      <c r="C405" s="90" t="s">
+      <c r="C405" s="93" t="s">
         <v>423</v>
       </c>
-      <c r="D405" s="90"/>
+      <c r="D405" s="93"/>
     </row>
     <row r="406" spans="2:38" ht="13.5" customHeight="1">
       <c r="B406" s="35" t="s">
         <v>424</v>
       </c>
-      <c r="C406" s="90" t="s">
+      <c r="C406" s="93" t="s">
         <v>425</v>
       </c>
-      <c r="D406" s="90"/>
+      <c r="D406" s="93"/>
     </row>
     <row r="407" spans="2:38" ht="13.5" customHeight="1">
       <c r="B407" s="35" t="s">
         <v>426</v>
       </c>
-      <c r="C407" s="90" t="s">
+      <c r="C407" s="93" t="s">
         <v>427</v>
       </c>
-      <c r="D407" s="90"/>
+      <c r="D407" s="93"/>
     </row>
     <row r="408" spans="2:38" ht="13.5" customHeight="1">
       <c r="B408" s="34"/>
@@ -30317,11 +30316,80 @@
     <row r="409" spans="2:38" ht="13.5" customHeight="1"/>
   </sheetData>
   <mergeCells count="95">
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="C62:D62"/>
-    <mergeCell ref="C75:D75"/>
-    <mergeCell ref="C79:D79"/>
-    <mergeCell ref="C102:D102"/>
+    <mergeCell ref="C228:D228"/>
+    <mergeCell ref="C268:D268"/>
+    <mergeCell ref="C309:D309"/>
+    <mergeCell ref="C306:D306"/>
+    <mergeCell ref="C292:D292"/>
+    <mergeCell ref="C291:D291"/>
+    <mergeCell ref="C244:D244"/>
+    <mergeCell ref="C270:D270"/>
+    <mergeCell ref="C296:D296"/>
+    <mergeCell ref="C294:D294"/>
+    <mergeCell ref="C304:D304"/>
+    <mergeCell ref="C301:D301"/>
+    <mergeCell ref="C299:D299"/>
+    <mergeCell ref="C234:D234"/>
+    <mergeCell ref="C229:D229"/>
+    <mergeCell ref="C407:D407"/>
+    <mergeCell ref="C406:D406"/>
+    <mergeCell ref="C405:D405"/>
+    <mergeCell ref="C337:D337"/>
+    <mergeCell ref="C335:D335"/>
+    <mergeCell ref="C351:D351"/>
+    <mergeCell ref="C348:D348"/>
+    <mergeCell ref="C346:D346"/>
+    <mergeCell ref="C404:D404"/>
+    <mergeCell ref="C403:D403"/>
+    <mergeCell ref="C384:D384"/>
+    <mergeCell ref="C379:D379"/>
+    <mergeCell ref="C372:D372"/>
+    <mergeCell ref="C370:D370"/>
+    <mergeCell ref="C367:D367"/>
+    <mergeCell ref="C365:D365"/>
+    <mergeCell ref="C375:D375"/>
+    <mergeCell ref="C362:D362"/>
+    <mergeCell ref="C396:D396"/>
+    <mergeCell ref="C390:D390"/>
+    <mergeCell ref="C386:D386"/>
+    <mergeCell ref="C394:D394"/>
+    <mergeCell ref="C315:D315"/>
+    <mergeCell ref="C331:D331"/>
+    <mergeCell ref="C242:D242"/>
+    <mergeCell ref="C289:D289"/>
+    <mergeCell ref="C281:D281"/>
+    <mergeCell ref="C279:D279"/>
+    <mergeCell ref="C277:D277"/>
+    <mergeCell ref="C275:D275"/>
+    <mergeCell ref="C257:D257"/>
+    <mergeCell ref="C255:D255"/>
+    <mergeCell ref="C253:D253"/>
+    <mergeCell ref="C251:D251"/>
+    <mergeCell ref="C247:D247"/>
+    <mergeCell ref="C249:D249"/>
+    <mergeCell ref="C285:D285"/>
+    <mergeCell ref="C287:D287"/>
+    <mergeCell ref="C231:D231"/>
+    <mergeCell ref="C237:D237"/>
+    <mergeCell ref="C240:D240"/>
+    <mergeCell ref="C167:D167"/>
+    <mergeCell ref="C202:D202"/>
+    <mergeCell ref="C213:D213"/>
+    <mergeCell ref="C215:D215"/>
+    <mergeCell ref="C217:D217"/>
+    <mergeCell ref="C173:D173"/>
+    <mergeCell ref="C179:D179"/>
+    <mergeCell ref="C190:D190"/>
+    <mergeCell ref="C193:D193"/>
+    <mergeCell ref="C198:D198"/>
+    <mergeCell ref="C196:D196"/>
+    <mergeCell ref="C220:D220"/>
+    <mergeCell ref="C225:D225"/>
+    <mergeCell ref="C130:D130"/>
+    <mergeCell ref="C134:D134"/>
+    <mergeCell ref="C137:D137"/>
+    <mergeCell ref="C139:D139"/>
+    <mergeCell ref="C144:D144"/>
     <mergeCell ref="C158:D158"/>
     <mergeCell ref="C162:D162"/>
     <mergeCell ref="C164:D164"/>
@@ -30338,80 +30406,11 @@
     <mergeCell ref="C40:D40"/>
     <mergeCell ref="C121:D121"/>
     <mergeCell ref="C93:D93"/>
-    <mergeCell ref="C130:D130"/>
-    <mergeCell ref="C134:D134"/>
-    <mergeCell ref="C137:D137"/>
-    <mergeCell ref="C139:D139"/>
-    <mergeCell ref="C144:D144"/>
-    <mergeCell ref="C231:D231"/>
-    <mergeCell ref="C237:D237"/>
-    <mergeCell ref="C240:D240"/>
-    <mergeCell ref="C167:D167"/>
-    <mergeCell ref="C202:D202"/>
-    <mergeCell ref="C213:D213"/>
-    <mergeCell ref="C215:D215"/>
-    <mergeCell ref="C217:D217"/>
-    <mergeCell ref="C173:D173"/>
-    <mergeCell ref="C179:D179"/>
-    <mergeCell ref="C190:D190"/>
-    <mergeCell ref="C193:D193"/>
-    <mergeCell ref="C198:D198"/>
-    <mergeCell ref="C196:D196"/>
-    <mergeCell ref="C220:D220"/>
-    <mergeCell ref="C315:D315"/>
-    <mergeCell ref="C331:D331"/>
-    <mergeCell ref="C242:D242"/>
-    <mergeCell ref="C289:D289"/>
-    <mergeCell ref="C281:D281"/>
-    <mergeCell ref="C279:D279"/>
-    <mergeCell ref="C277:D277"/>
-    <mergeCell ref="C275:D275"/>
-    <mergeCell ref="C257:D257"/>
-    <mergeCell ref="C255:D255"/>
-    <mergeCell ref="C253:D253"/>
-    <mergeCell ref="C251:D251"/>
-    <mergeCell ref="C247:D247"/>
-    <mergeCell ref="C249:D249"/>
-    <mergeCell ref="C285:D285"/>
-    <mergeCell ref="C287:D287"/>
-    <mergeCell ref="C375:D375"/>
-    <mergeCell ref="C362:D362"/>
-    <mergeCell ref="C396:D396"/>
-    <mergeCell ref="C390:D390"/>
-    <mergeCell ref="C386:D386"/>
-    <mergeCell ref="C394:D394"/>
-    <mergeCell ref="C407:D407"/>
-    <mergeCell ref="C406:D406"/>
-    <mergeCell ref="C405:D405"/>
-    <mergeCell ref="C337:D337"/>
-    <mergeCell ref="C335:D335"/>
-    <mergeCell ref="C351:D351"/>
-    <mergeCell ref="C348:D348"/>
-    <mergeCell ref="C346:D346"/>
-    <mergeCell ref="C404:D404"/>
-    <mergeCell ref="C403:D403"/>
-    <mergeCell ref="C384:D384"/>
-    <mergeCell ref="C379:D379"/>
-    <mergeCell ref="C372:D372"/>
-    <mergeCell ref="C370:D370"/>
-    <mergeCell ref="C367:D367"/>
-    <mergeCell ref="C365:D365"/>
-    <mergeCell ref="C225:D225"/>
-    <mergeCell ref="C228:D228"/>
-    <mergeCell ref="C268:D268"/>
-    <mergeCell ref="C309:D309"/>
-    <mergeCell ref="C306:D306"/>
-    <mergeCell ref="C292:D292"/>
-    <mergeCell ref="C291:D291"/>
-    <mergeCell ref="C244:D244"/>
-    <mergeCell ref="C270:D270"/>
-    <mergeCell ref="C296:D296"/>
-    <mergeCell ref="C294:D294"/>
-    <mergeCell ref="C304:D304"/>
-    <mergeCell ref="C301:D301"/>
-    <mergeCell ref="C299:D299"/>
-    <mergeCell ref="C234:D234"/>
-    <mergeCell ref="C229:D229"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C62:D62"/>
+    <mergeCell ref="C75:D75"/>
+    <mergeCell ref="C79:D79"/>
+    <mergeCell ref="C102:D102"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.39370078740157483" bottom="0" header="0" footer="0"/>
@@ -30433,15 +30432,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A26:K40"/>
-  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.44140625" customWidth="1"/>
-    <col min="2" max="2" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="2" max="2" width="7.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="10" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="10" width="7.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="5.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="26" spans="1:11">
@@ -30759,49 +30758,49 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:P59"/>
-  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="13.44140625" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.6">
-      <c r="A1" s="104" t="s">
+    <row r="1" spans="1:15" ht="15.75">
+      <c r="A1" s="96" t="s">
         <v>441</v>
       </c>
-      <c r="B1" s="104"/>
-      <c r="C1" s="104"/>
-      <c r="D1" s="104"/>
-      <c r="E1" s="104"/>
-      <c r="F1" s="104"/>
-      <c r="G1" s="104"/>
+      <c r="B1" s="96"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
       <c r="H1" s="9"/>
-      <c r="I1" s="101" t="s">
+      <c r="I1" s="97" t="s">
         <v>442</v>
       </c>
-      <c r="J1" s="101"/>
-      <c r="K1" s="101"/>
-      <c r="L1" s="101"/>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
-      <c r="O1" s="101"/>
-    </row>
-    <row r="2" spans="1:15" ht="15.6">
-      <c r="A2" s="104"/>
-      <c r="B2" s="104"/>
-      <c r="C2" s="104"/>
-      <c r="D2" s="104"/>
-      <c r="E2" s="104"/>
-      <c r="F2" s="104"/>
-      <c r="G2" s="104"/>
+      <c r="J1" s="97"/>
+      <c r="K1" s="97"/>
+      <c r="L1" s="97"/>
+      <c r="M1" s="97"/>
+      <c r="N1" s="97"/>
+      <c r="O1" s="97"/>
+    </row>
+    <row r="2" spans="1:15" ht="15.75">
+      <c r="A2" s="96"/>
+      <c r="B2" s="96"/>
+      <c r="C2" s="96"/>
+      <c r="D2" s="96"/>
+      <c r="E2" s="96"/>
+      <c r="F2" s="96"/>
+      <c r="G2" s="96"/>
       <c r="H2" s="9"/>
-      <c r="I2" s="101"/>
-      <c r="J2" s="101"/>
-      <c r="K2" s="101"/>
-      <c r="L2" s="101"/>
-      <c r="M2" s="101"/>
-      <c r="N2" s="101"/>
-      <c r="O2" s="101"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="97"/>
+      <c r="K2" s="97"/>
+      <c r="L2" s="97"/>
+      <c r="M2" s="97"/>
+      <c r="N2" s="97"/>
+      <c r="O2" s="97"/>
     </row>
     <row r="3" spans="1:15">
       <c r="A3" s="98" t="s">
@@ -30841,15 +30840,15 @@
       <c r="N4" s="98"/>
       <c r="O4" s="98"/>
     </row>
-    <row r="5" spans="1:15" ht="41.4">
-      <c r="A5" s="100" t="s">
+    <row r="5" spans="1:15" ht="38.25">
+      <c r="A5" s="99" t="s">
         <v>445</v>
       </c>
-      <c r="B5" s="100"/>
-      <c r="C5" s="100" t="s">
+      <c r="B5" s="99"/>
+      <c r="C5" s="99" t="s">
         <v>446</v>
       </c>
-      <c r="D5" s="100" t="s">
+      <c r="D5" s="99" t="s">
         <v>447</v>
       </c>
       <c r="E5" s="12" t="s">
@@ -30861,23 +30860,23 @@
       <c r="G5" s="12" t="s">
         <v>450</v>
       </c>
-      <c r="I5" s="100" t="s">
+      <c r="I5" s="99" t="s">
         <v>445</v>
       </c>
-      <c r="J5" s="100"/>
-      <c r="K5" s="100" t="s">
+      <c r="J5" s="99"/>
+      <c r="K5" s="99" t="s">
         <v>451</v>
       </c>
-      <c r="L5" s="100"/>
-      <c r="M5" s="100"/>
-      <c r="N5" s="100"/>
-      <c r="O5" s="100"/>
-    </row>
-    <row r="6" spans="1:15" ht="42.6">
-      <c r="A6" s="100"/>
-      <c r="B6" s="100"/>
-      <c r="C6" s="100"/>
-      <c r="D6" s="100"/>
+      <c r="L5" s="99"/>
+      <c r="M5" s="99"/>
+      <c r="N5" s="99"/>
+      <c r="O5" s="99"/>
+    </row>
+    <row r="6" spans="1:15" ht="40.5">
+      <c r="A6" s="99"/>
+      <c r="B6" s="99"/>
+      <c r="C6" s="99"/>
+      <c r="D6" s="99"/>
       <c r="E6" s="12" t="s">
         <v>452</v>
       </c>
@@ -30887,12 +30886,12 @@
       <c r="G6" s="12" t="s">
         <v>454</v>
       </c>
-      <c r="I6" s="100"/>
-      <c r="J6" s="100"/>
-      <c r="K6" s="100" t="s">
+      <c r="I6" s="99"/>
+      <c r="J6" s="99"/>
+      <c r="K6" s="99" t="s">
         <v>455</v>
       </c>
-      <c r="L6" s="100" t="s">
+      <c r="L6" s="99" t="s">
         <v>456</v>
       </c>
       <c r="M6" s="12" t="s">
@@ -30905,7 +30904,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="27.6">
+    <row r="7" spans="1:15" ht="25.5">
       <c r="A7" s="19">
         <v>2016</v>
       </c>
@@ -30930,10 +30929,10 @@
         <f>SUM(G8:G19)*1000</f>
         <v>1169544759</v>
       </c>
-      <c r="I7" s="100"/>
-      <c r="J7" s="100"/>
-      <c r="K7" s="100"/>
-      <c r="L7" s="100"/>
+      <c r="I7" s="99"/>
+      <c r="J7" s="99"/>
+      <c r="K7" s="99"/>
+      <c r="L7" s="99"/>
       <c r="M7" s="12" t="s">
         <v>458</v>
       </c>
@@ -31433,14 +31432,14 @@
       <c r="A20" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="B20" s="99" t="s">
+      <c r="B20" s="100" t="s">
         <v>473</v>
       </c>
-      <c r="C20" s="99"/>
-      <c r="D20" s="99"/>
-      <c r="E20" s="99"/>
-      <c r="F20" s="99"/>
-      <c r="G20" s="99"/>
+      <c r="C20" s="100"/>
+      <c r="D20" s="100"/>
+      <c r="E20" s="100"/>
+      <c r="F20" s="100"/>
+      <c r="G20" s="100"/>
       <c r="I20" s="98" t="s">
         <v>472</v>
       </c>
@@ -31461,221 +31460,221 @@
         <v>7569.8</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="15">
+    <row r="21" spans="1:16">
       <c r="A21" s="15" t="s">
         <v>474</v>
       </c>
-      <c r="B21" s="99" t="s">
+      <c r="B21" s="100" t="s">
         <v>475</v>
       </c>
-      <c r="C21" s="99"/>
-      <c r="D21" s="99"/>
-      <c r="E21" s="99"/>
-      <c r="F21" s="99"/>
-      <c r="G21" s="99"/>
-      <c r="I21" s="103" t="s">
+      <c r="C21" s="100"/>
+      <c r="D21" s="100"/>
+      <c r="E21" s="100"/>
+      <c r="F21" s="100"/>
+      <c r="G21" s="100"/>
+      <c r="I21" s="101" t="s">
         <v>71</v>
       </c>
-      <c r="J21" s="99" t="s">
+      <c r="J21" s="100" t="s">
         <v>476</v>
       </c>
-      <c r="K21" s="99"/>
-      <c r="L21" s="99"/>
-      <c r="M21" s="99"/>
-      <c r="N21" s="99"/>
-      <c r="O21" s="99"/>
-    </row>
-    <row r="22" spans="1:16" ht="15">
+      <c r="K21" s="100"/>
+      <c r="L21" s="100"/>
+      <c r="M21" s="100"/>
+      <c r="N21" s="100"/>
+      <c r="O21" s="100"/>
+    </row>
+    <row r="22" spans="1:16">
       <c r="A22" s="15" t="s">
         <v>477</v>
       </c>
-      <c r="B22" s="99" t="s">
+      <c r="B22" s="100" t="s">
         <v>478</v>
       </c>
-      <c r="C22" s="99"/>
-      <c r="D22" s="99"/>
-      <c r="E22" s="99"/>
-      <c r="F22" s="99"/>
-      <c r="G22" s="99"/>
-      <c r="I22" s="103"/>
-      <c r="J22" s="99" t="s">
+      <c r="C22" s="100"/>
+      <c r="D22" s="100"/>
+      <c r="E22" s="100"/>
+      <c r="F22" s="100"/>
+      <c r="G22" s="100"/>
+      <c r="I22" s="101"/>
+      <c r="J22" s="100" t="s">
         <v>479</v>
       </c>
-      <c r="K22" s="99"/>
-      <c r="L22" s="99"/>
-      <c r="M22" s="99"/>
-      <c r="N22" s="99"/>
-      <c r="O22" s="99"/>
-    </row>
-    <row r="23" spans="1:16" ht="15">
+      <c r="K22" s="100"/>
+      <c r="L22" s="100"/>
+      <c r="M22" s="100"/>
+      <c r="N22" s="100"/>
+      <c r="O22" s="100"/>
+    </row>
+    <row r="23" spans="1:16">
       <c r="A23" s="15" t="s">
         <v>480</v>
       </c>
-      <c r="B23" s="99" t="s">
+      <c r="B23" s="100" t="s">
         <v>481</v>
       </c>
-      <c r="C23" s="99"/>
-      <c r="D23" s="99"/>
-      <c r="E23" s="99"/>
-      <c r="F23" s="99"/>
-      <c r="G23" s="99"/>
+      <c r="C23" s="100"/>
+      <c r="D23" s="100"/>
+      <c r="E23" s="100"/>
+      <c r="F23" s="100"/>
+      <c r="G23" s="100"/>
       <c r="I23" s="15" t="s">
         <v>474</v>
       </c>
-      <c r="J23" s="99" t="s">
+      <c r="J23" s="100" t="s">
         <v>475</v>
       </c>
-      <c r="K23" s="99"/>
-      <c r="L23" s="99"/>
-      <c r="M23" s="99"/>
-      <c r="N23" s="99"/>
-      <c r="O23" s="99"/>
-    </row>
-    <row r="24" spans="1:16" ht="15">
+      <c r="K23" s="100"/>
+      <c r="L23" s="100"/>
+      <c r="M23" s="100"/>
+      <c r="N23" s="100"/>
+      <c r="O23" s="100"/>
+    </row>
+    <row r="24" spans="1:16">
       <c r="A24" s="15" t="s">
         <v>482</v>
       </c>
-      <c r="B24" s="99" t="s">
+      <c r="B24" s="100" t="s">
         <v>483</v>
       </c>
-      <c r="C24" s="99"/>
-      <c r="D24" s="99"/>
-      <c r="E24" s="99"/>
-      <c r="F24" s="99"/>
-      <c r="G24" s="99"/>
+      <c r="C24" s="100"/>
+      <c r="D24" s="100"/>
+      <c r="E24" s="100"/>
+      <c r="F24" s="100"/>
+      <c r="G24" s="100"/>
       <c r="I24" s="15" t="s">
         <v>477</v>
       </c>
-      <c r="J24" s="99" t="s">
+      <c r="J24" s="100" t="s">
         <v>484</v>
       </c>
-      <c r="K24" s="99"/>
-      <c r="L24" s="99"/>
-      <c r="M24" s="99"/>
-      <c r="N24" s="99"/>
-      <c r="O24" s="99"/>
-    </row>
-    <row r="25" spans="1:16" ht="15">
+      <c r="K24" s="100"/>
+      <c r="L24" s="100"/>
+      <c r="M24" s="100"/>
+      <c r="N24" s="100"/>
+      <c r="O24" s="100"/>
+    </row>
+    <row r="25" spans="1:16">
       <c r="A25" s="15" t="s">
         <v>485</v>
       </c>
-      <c r="B25" s="99" t="s">
+      <c r="B25" s="100" t="s">
         <v>486</v>
       </c>
-      <c r="C25" s="99"/>
-      <c r="D25" s="99"/>
-      <c r="E25" s="99"/>
-      <c r="F25" s="99"/>
-      <c r="G25" s="99"/>
-      <c r="I25" s="96"/>
-      <c r="J25" s="96"/>
+      <c r="C25" s="100"/>
+      <c r="D25" s="100"/>
+      <c r="E25" s="100"/>
+      <c r="F25" s="100"/>
+      <c r="G25" s="100"/>
+      <c r="I25" s="102"/>
+      <c r="J25" s="102"/>
     </row>
     <row r="26" spans="1:16">
-      <c r="A26" s="97" t="s">
+      <c r="A26" s="103" t="s">
         <v>487</v>
       </c>
-      <c r="B26" s="97"/>
-      <c r="I26" s="97" t="s">
+      <c r="B26" s="103"/>
+      <c r="I26" s="103" t="s">
         <v>487</v>
       </c>
-      <c r="J26" s="97"/>
+      <c r="J26" s="103"/>
     </row>
     <row r="28" spans="1:16">
-      <c r="A28" s="101" t="s">
+      <c r="A28" s="97" t="s">
         <v>488</v>
       </c>
-      <c r="B28" s="101"/>
-      <c r="C28" s="101"/>
-      <c r="D28" s="101"/>
-      <c r="E28" s="101"/>
-      <c r="F28" s="101"/>
-      <c r="G28" s="101"/>
-      <c r="I28" s="101" t="s">
+      <c r="B28" s="97"/>
+      <c r="C28" s="97"/>
+      <c r="D28" s="97"/>
+      <c r="E28" s="97"/>
+      <c r="F28" s="97"/>
+      <c r="G28" s="97"/>
+      <c r="I28" s="97" t="s">
         <v>489</v>
       </c>
-      <c r="J28" s="101"/>
-      <c r="K28" s="101"/>
-      <c r="L28" s="101"/>
-      <c r="M28" s="101"/>
-      <c r="N28" s="101"/>
-      <c r="O28" s="101"/>
-      <c r="P28" s="101"/>
+      <c r="J28" s="97"/>
+      <c r="K28" s="97"/>
+      <c r="L28" s="97"/>
+      <c r="M28" s="97"/>
+      <c r="N28" s="97"/>
+      <c r="O28" s="97"/>
+      <c r="P28" s="97"/>
     </row>
     <row r="29" spans="1:16">
-      <c r="A29" s="101"/>
-      <c r="B29" s="101"/>
-      <c r="C29" s="101"/>
-      <c r="D29" s="101"/>
-      <c r="E29" s="101"/>
-      <c r="F29" s="101"/>
-      <c r="G29" s="101"/>
-      <c r="I29" s="101"/>
-      <c r="J29" s="101"/>
-      <c r="K29" s="101"/>
-      <c r="L29" s="101"/>
-      <c r="M29" s="101"/>
-      <c r="N29" s="101"/>
-      <c r="O29" s="101"/>
-      <c r="P29" s="101"/>
+      <c r="A29" s="97"/>
+      <c r="B29" s="97"/>
+      <c r="C29" s="97"/>
+      <c r="D29" s="97"/>
+      <c r="E29" s="97"/>
+      <c r="F29" s="97"/>
+      <c r="G29" s="97"/>
+      <c r="I29" s="97"/>
+      <c r="J29" s="97"/>
+      <c r="K29" s="97"/>
+      <c r="L29" s="97"/>
+      <c r="M29" s="97"/>
+      <c r="N29" s="97"/>
+      <c r="O29" s="97"/>
+      <c r="P29" s="97"/>
     </row>
     <row r="30" spans="1:16">
-      <c r="A30" s="102" t="s">
+      <c r="A30" s="104" t="s">
         <v>490</v>
       </c>
-      <c r="B30" s="102"/>
-      <c r="C30" s="102"/>
-      <c r="D30" s="102"/>
-      <c r="E30" s="102"/>
-      <c r="F30" s="102"/>
-      <c r="G30" s="102"/>
-      <c r="I30" s="102" t="s">
+      <c r="B30" s="104"/>
+      <c r="C30" s="104"/>
+      <c r="D30" s="104"/>
+      <c r="E30" s="104"/>
+      <c r="F30" s="104"/>
+      <c r="G30" s="104"/>
+      <c r="I30" s="104" t="s">
         <v>491</v>
       </c>
-      <c r="J30" s="102"/>
-      <c r="K30" s="102"/>
-      <c r="L30" s="102"/>
-      <c r="M30" s="102"/>
-      <c r="N30" s="102"/>
-      <c r="O30" s="102"/>
-      <c r="P30" s="102"/>
+      <c r="J30" s="104"/>
+      <c r="K30" s="104"/>
+      <c r="L30" s="104"/>
+      <c r="M30" s="104"/>
+      <c r="N30" s="104"/>
+      <c r="O30" s="104"/>
+      <c r="P30" s="104"/>
     </row>
     <row r="31" spans="1:16">
-      <c r="A31" s="96"/>
-      <c r="B31" s="96"/>
-      <c r="C31" s="96"/>
-      <c r="D31" s="96"/>
-      <c r="E31" s="96"/>
-      <c r="F31" s="96"/>
-      <c r="G31" s="96"/>
-      <c r="I31" s="96"/>
-      <c r="J31" s="96"/>
-      <c r="K31" s="96"/>
-      <c r="L31" s="96"/>
-      <c r="M31" s="96"/>
-      <c r="N31" s="96"/>
-      <c r="O31" s="96"/>
-      <c r="P31" s="96"/>
-    </row>
-    <row r="32" spans="1:16" ht="41.4">
-      <c r="A32" s="100" t="s">
+      <c r="A31" s="102"/>
+      <c r="B31" s="102"/>
+      <c r="C31" s="102"/>
+      <c r="D31" s="102"/>
+      <c r="E31" s="102"/>
+      <c r="F31" s="102"/>
+      <c r="G31" s="102"/>
+      <c r="I31" s="102"/>
+      <c r="J31" s="102"/>
+      <c r="K31" s="102"/>
+      <c r="L31" s="102"/>
+      <c r="M31" s="102"/>
+      <c r="N31" s="102"/>
+      <c r="O31" s="102"/>
+      <c r="P31" s="102"/>
+    </row>
+    <row r="32" spans="1:16" ht="38.25">
+      <c r="A32" s="99" t="s">
         <v>445</v>
       </c>
-      <c r="B32" s="100"/>
-      <c r="C32" s="100" t="s">
+      <c r="B32" s="99"/>
+      <c r="C32" s="99" t="s">
         <v>492</v>
       </c>
-      <c r="D32" s="100"/>
-      <c r="E32" s="100"/>
-      <c r="F32" s="100"/>
-      <c r="G32" s="100"/>
-      <c r="I32" s="100" t="s">
+      <c r="D32" s="99"/>
+      <c r="E32" s="99"/>
+      <c r="F32" s="99"/>
+      <c r="G32" s="99"/>
+      <c r="I32" s="99" t="s">
         <v>445</v>
       </c>
-      <c r="J32" s="100"/>
+      <c r="J32" s="99"/>
       <c r="K32" s="12" t="s">
         <v>493</v>
       </c>
-      <c r="L32" s="100" t="s">
+      <c r="L32" s="99" t="s">
         <v>494</v>
       </c>
       <c r="M32" s="12" t="s">
@@ -31691,13 +31690,13 @@
         <v>495</v>
       </c>
     </row>
-    <row r="33" spans="1:16" ht="41.4">
-      <c r="A33" s="100"/>
-      <c r="B33" s="100"/>
-      <c r="C33" s="100" t="s">
+    <row r="33" spans="1:16" ht="38.25">
+      <c r="A33" s="99"/>
+      <c r="B33" s="99"/>
+      <c r="C33" s="99" t="s">
         <v>455</v>
       </c>
-      <c r="D33" s="100" t="s">
+      <c r="D33" s="99" t="s">
         <v>456</v>
       </c>
       <c r="E33" s="12" t="s">
@@ -31709,12 +31708,12 @@
       <c r="G33" s="12" t="s">
         <v>457</v>
       </c>
-      <c r="I33" s="100"/>
-      <c r="J33" s="100"/>
+      <c r="I33" s="99"/>
+      <c r="J33" s="99"/>
       <c r="K33" s="12" t="s">
         <v>496</v>
       </c>
-      <c r="L33" s="100"/>
+      <c r="L33" s="99"/>
       <c r="M33" s="12" t="s">
         <v>497</v>
       </c>
@@ -31728,11 +31727,11 @@
         <v>498</v>
       </c>
     </row>
-    <row r="34" spans="1:16" ht="27.6">
-      <c r="A34" s="100"/>
-      <c r="B34" s="100"/>
-      <c r="C34" s="100"/>
-      <c r="D34" s="100"/>
+    <row r="34" spans="1:16" ht="25.5">
+      <c r="A34" s="99"/>
+      <c r="B34" s="99"/>
+      <c r="C34" s="99"/>
+      <c r="D34" s="99"/>
       <c r="E34" s="12" t="s">
         <v>497</v>
       </c>
@@ -32292,7 +32291,7 @@
         <v>3378.7449999999999</v>
       </c>
     </row>
-    <row r="47" spans="1:16" ht="15">
+    <row r="47" spans="1:16">
       <c r="A47" s="98" t="s">
         <v>472</v>
       </c>
@@ -32315,69 +32314,69 @@
       <c r="I47" s="15" t="s">
         <v>474</v>
       </c>
-      <c r="J47" s="99" t="s">
+      <c r="J47" s="100" t="s">
         <v>475</v>
       </c>
-      <c r="K47" s="99"/>
-      <c r="L47" s="99"/>
-      <c r="M47" s="99"/>
-      <c r="N47" s="99"/>
-      <c r="O47" s="99"/>
-      <c r="P47" s="99"/>
-    </row>
-    <row r="48" spans="1:16" ht="15">
+      <c r="K47" s="100"/>
+      <c r="L47" s="100"/>
+      <c r="M47" s="100"/>
+      <c r="N47" s="100"/>
+      <c r="O47" s="100"/>
+      <c r="P47" s="100"/>
+    </row>
+    <row r="48" spans="1:16">
       <c r="A48" s="15" t="s">
         <v>474</v>
       </c>
-      <c r="B48" s="99" t="s">
+      <c r="B48" s="100" t="s">
         <v>475</v>
       </c>
-      <c r="C48" s="99"/>
-      <c r="D48" s="99"/>
-      <c r="E48" s="99"/>
-      <c r="F48" s="99"/>
-      <c r="G48" s="99"/>
+      <c r="C48" s="100"/>
+      <c r="D48" s="100"/>
+      <c r="E48" s="100"/>
+      <c r="F48" s="100"/>
+      <c r="G48" s="100"/>
       <c r="I48" s="15" t="s">
         <v>477</v>
       </c>
-      <c r="J48" s="99" t="s">
+      <c r="J48" s="100" t="s">
         <v>499</v>
       </c>
-      <c r="K48" s="99"/>
-      <c r="L48" s="99"/>
-      <c r="M48" s="99"/>
-      <c r="N48" s="99"/>
-      <c r="O48" s="99"/>
-      <c r="P48" s="99"/>
-    </row>
-    <row r="49" spans="1:10" ht="15">
+      <c r="K48" s="100"/>
+      <c r="L48" s="100"/>
+      <c r="M48" s="100"/>
+      <c r="N48" s="100"/>
+      <c r="O48" s="100"/>
+      <c r="P48" s="100"/>
+    </row>
+    <row r="49" spans="1:10">
       <c r="A49" s="15" t="s">
         <v>477</v>
       </c>
-      <c r="B49" s="99" t="s">
+      <c r="B49" s="100" t="s">
         <v>484</v>
       </c>
-      <c r="C49" s="99"/>
-      <c r="D49" s="99"/>
-      <c r="E49" s="99"/>
-      <c r="F49" s="99"/>
-      <c r="G49" s="99"/>
-      <c r="I49" s="96"/>
-      <c r="J49" s="96"/>
+      <c r="C49" s="100"/>
+      <c r="D49" s="100"/>
+      <c r="E49" s="100"/>
+      <c r="F49" s="100"/>
+      <c r="G49" s="100"/>
+      <c r="I49" s="102"/>
+      <c r="J49" s="102"/>
     </row>
     <row r="50" spans="1:10" ht="37.5" customHeight="1">
-      <c r="A50" s="96"/>
-      <c r="B50" s="96"/>
-      <c r="I50" s="97" t="s">
+      <c r="A50" s="102"/>
+      <c r="B50" s="102"/>
+      <c r="I50" s="103" t="s">
         <v>487</v>
       </c>
-      <c r="J50" s="97"/>
+      <c r="J50" s="103"/>
     </row>
     <row r="51" spans="1:10" ht="33" customHeight="1">
-      <c r="A51" s="97" t="s">
+      <c r="A51" s="103" t="s">
         <v>487</v>
       </c>
-      <c r="B51" s="97"/>
+      <c r="B51" s="103"/>
     </row>
     <row r="54" spans="1:10" ht="33.75" customHeight="1">
       <c r="C54" s="16" t="s">
@@ -32434,6 +32433,88 @@
     </row>
   </sheetData>
   <mergeCells count="93">
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="I50:J50"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="J47:P47"/>
+    <mergeCell ref="B48:G48"/>
+    <mergeCell ref="J48:P48"/>
+    <mergeCell ref="B49:G49"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="I39:J39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="I31:P31"/>
+    <mergeCell ref="A32:B34"/>
+    <mergeCell ref="C32:G32"/>
+    <mergeCell ref="I32:J33"/>
+    <mergeCell ref="L32:L33"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="A28:G29"/>
+    <mergeCell ref="I28:P29"/>
+    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="I30:P30"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="J23:O23"/>
+    <mergeCell ref="B24:G24"/>
+    <mergeCell ref="J24:O24"/>
+    <mergeCell ref="B25:G25"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="J21:O21"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="J22:O22"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="I10:J10"/>
     <mergeCell ref="A1:G2"/>
     <mergeCell ref="I1:O2"/>
     <mergeCell ref="A3:G4"/>
@@ -32445,88 +32526,6 @@
     <mergeCell ref="K5:O5"/>
     <mergeCell ref="K6:K7"/>
     <mergeCell ref="L6:L7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="B20:G20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="J21:O21"/>
-    <mergeCell ref="B22:G22"/>
-    <mergeCell ref="J22:O22"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="J23:O23"/>
-    <mergeCell ref="B24:G24"/>
-    <mergeCell ref="J24:O24"/>
-    <mergeCell ref="B25:G25"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="A28:G29"/>
-    <mergeCell ref="I28:P29"/>
-    <mergeCell ref="A30:G30"/>
-    <mergeCell ref="I30:P30"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="I31:P31"/>
-    <mergeCell ref="A32:B34"/>
-    <mergeCell ref="C32:G32"/>
-    <mergeCell ref="I32:J33"/>
-    <mergeCell ref="L32:L33"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="I38:J38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="I39:J39"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="I42:J42"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="I44:J44"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="I46:J46"/>
-    <mergeCell ref="A50:B50"/>
-    <mergeCell ref="I50:J50"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="J47:P47"/>
-    <mergeCell ref="B48:G48"/>
-    <mergeCell ref="J48:P48"/>
-    <mergeCell ref="B49:G49"/>
-    <mergeCell ref="I49:J49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -32535,7 +32534,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A2:R338"/>
-  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
   </cols>
@@ -32585,7 +32584,7 @@
         <v>382.92</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15.6">
+    <row r="13" spans="1:3" ht="15.75">
       <c r="A13" s="27" t="s">
         <v>512</v>
       </c>
@@ -32600,7 +32599,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="303.60000000000002">
+    <row r="17" spans="1:18" ht="293.25">
       <c r="A17" s="30" t="s">
         <v>515</v>
       </c>
@@ -49828,16 +49827,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A335:R335"/>
-    <mergeCell ref="A336:R336"/>
-    <mergeCell ref="A337:R337"/>
-    <mergeCell ref="A338:R338"/>
-    <mergeCell ref="A329:R329"/>
-    <mergeCell ref="A330:R330"/>
-    <mergeCell ref="A331:R331"/>
-    <mergeCell ref="A332:R332"/>
-    <mergeCell ref="A333:R333"/>
-    <mergeCell ref="A334:R334"/>
     <mergeCell ref="A328:R328"/>
     <mergeCell ref="A317:R317"/>
     <mergeCell ref="A318:R318"/>
@@ -49850,6 +49839,16 @@
     <mergeCell ref="A325:R325"/>
     <mergeCell ref="A326:R326"/>
     <mergeCell ref="A327:R327"/>
+    <mergeCell ref="A335:R335"/>
+    <mergeCell ref="A336:R336"/>
+    <mergeCell ref="A337:R337"/>
+    <mergeCell ref="A338:R338"/>
+    <mergeCell ref="A329:R329"/>
+    <mergeCell ref="A330:R330"/>
+    <mergeCell ref="A331:R331"/>
+    <mergeCell ref="A332:R332"/>
+    <mergeCell ref="A333:R333"/>
+    <mergeCell ref="A334:R334"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B7" r:id="rId1" xr:uid="{CEA94E12-8357-E942-8D00-C6277BD2893C}"/>
@@ -49864,13 +49863,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.88671875" customWidth="1"/>
-    <col min="2" max="8" width="10.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" customWidth="1"/>
+    <col min="2" max="8" width="10.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.8">
+    <row r="1" spans="1:8" ht="30">
       <c r="A1" s="23" t="s">
         <v>97</v>
       </c>
@@ -50086,13 +50085,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:H12"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.88671875" customWidth="1"/>
-    <col min="2" max="8" width="10.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" customWidth="1"/>
+    <col min="2" max="8" width="10.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.8">
+    <row r="1" spans="1:8" ht="30">
       <c r="A1" s="23" t="s">
         <v>97</v>
       </c>
@@ -50132,11 +50131,11 @@
       </c>
       <c r="D2" s="87">
         <f>RoadTransport!D71</f>
-        <v>1747052.7753335293</v>
+        <v>26255.622243626291</v>
       </c>
       <c r="E2" s="87">
         <f>RoadTransport!E71</f>
-        <v>32422.84691009732</v>
+        <v>1753220</v>
       </c>
       <c r="F2" s="87">
         <f>RoadTransport!F71</f>
@@ -50165,11 +50164,11 @@
       </c>
       <c r="D3" s="87">
         <f>RoadTransport!D72</f>
-        <v>606439.22497603227</v>
+        <v>9113.8856418624528</v>
       </c>
       <c r="E3" s="87">
         <f>RoadTransport!E72</f>
-        <v>11254.660665830315</v>
+        <v>608580</v>
       </c>
       <c r="F3" s="87">
         <f>RoadTransport!F72</f>
@@ -50342,15 +50341,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
     <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
@@ -50494,6 +50484,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -50501,14 +50500,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CA6F3F9-54E8-42CE-BA1E-720513583380}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0111859B-CD30-4769-AFDE-679195CD6BDD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -50526,6 +50517,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2CA6F3F9-54E8-42CE-BA1E-720513583380}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{33C1B47E-950D-4DFF-9560-C2E26531F87C}">
   <ds:schemaRefs>

</xml_diff>